<commit_message>
Add Bugs sheet to UAT report and email draft
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KaHijVTfXKJr6MMzYd7aP
</commit_message>
<xml_diff>
--- a/Protec_UAT_API_Test_Report.xlsx
+++ b/Protec_UAT_API_Test_Report.xlsx
@@ -8,18 +8,19 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All APIs" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Success" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Failure" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocked" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not tested" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bugs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All APIs" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Success" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Failure" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Blocked" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not tested" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'All APIs'!$A$1:$K$86</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Success'!$A$1:$K$81</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Failure'!$A$1:$K$6</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Blocked'!$A$1:$K$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Not tested'!$A$1:$K$5</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All APIs'!$A$1:$K$86</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Success'!$A$1:$K$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Failure'!$A$1:$K$6</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Blocked'!$A$1:$K$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Not tested'!$A$1:$K$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -45,7 +46,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="8">
+  <fills count="9">
     <fill>
       <patternFill/>
     </fill>
@@ -82,6 +83,11 @@
         <fgColor rgb="00305496"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -95,7 +101,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -119,6 +125,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -765,6 +774,396 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:J7"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="9" customWidth="1" min="2" max="2"/>
+    <col width="30" customWidth="1" min="3" max="3"/>
+    <col width="44" customWidth="1" min="4" max="4"/>
+    <col width="50" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="50" customWidth="1" min="8" max="8"/>
+    <col width="44" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="13" t="inlineStr">
+        <is>
+          <t>Bug ID</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>Severity</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>API / use case</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="E1" s="13" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+      <c r="F1" s="13" t="inlineStr">
+        <is>
+          <t>Steps to reproduce</t>
+        </is>
+      </c>
+      <c r="G1" s="13" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="H1" s="13" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="I1" s="13" t="inlineStr">
+        <is>
+          <t>Evidence (trace / policy / claim)</t>
+        </is>
+      </c>
+      <c r="J1" s="13" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="8" t="inlineStr">
+        <is>
+          <t>UAT-BUG-01</t>
+        </is>
+      </c>
+      <c r="B2" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C2" s="8" t="inlineStr">
+        <is>
+          <t>A31.1 proposalSendPrepayment (float issuance)</t>
+        </is>
+      </c>
+      <c r="D2" s="8" t="inlineStr">
+        <is>
+          <t>POST /api/protecuat/api-orchestration/v1/flow/agentPortal_proposalSendPrepayment</t>
+        </is>
+      </c>
+      <c r="E2" s="8" t="inlineStr">
+        <is>
+          <t>Policy issued on float with NO float debit when underwriting result is a referral (AutoUwResultCode 2)</t>
+        </is>
+      </c>
+      <c r="F2" s="8" t="inlineStr">
+        <is>
+          <t>1) Agent PTY00000000000003 with float 532527. 2) Quote/bind PCAR with VehicleMake 1001 (UW referral) or PCV with RTO MH12. 3) Call proposalSendPrepayment with the bound PolicyObject.</t>
+        </is>
+      </c>
+      <c r="G2" s="8" t="inlineStr">
+        <is>
+          <t>Either float debited by DuePremium, or policy not issued until UW approves.</t>
+        </is>
+      </c>
+      <c r="H2" s="8" t="inlineStr">
+        <is>
+          <t>Policy reaches ProposalStatus 3 (issued) and getCollectionTransHis shows no debit. Same PCAR with make 1002 (AutoUwResultCode 1) is debited 4473.38.</t>
+        </is>
+      </c>
+      <c r="I2" s="8" t="inlineStr">
+        <is>
+          <t>PP-1005-26-00000052-00 (4473.38) and PP-1202-26-00000027-00 (27358.30) not debited; PP-1005-26-00000053-00 debited</t>
+        </is>
+      </c>
+      <c r="J2" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="8" t="inlineStr">
+        <is>
+          <t>UAT-BUG-02</t>
+        </is>
+      </c>
+      <c r="B3" s="8" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="C3" s="8" t="inlineStr">
+        <is>
+          <t>A27.1 proposalValidate / A29.1 proposalBind</t>
+        </is>
+      </c>
+      <c r="D3" s="8" t="inlineStr">
+        <is>
+          <t>POST .../agentPortal_proposalValidate and .../agentPortal_proposalBind</t>
+        </is>
+      </c>
+      <c r="E3" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 500 for registered vehicles (MH12AB1234, KA01AB1234); same proposals pass with MH12XX0008 or RegistrationNo NEW</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
+          <t>1) Persist/calc/create/save/calc a P2W (or PCV/GCV) proposal with RegistrationNo MH12AB1234, ChannelType AP. 2) Call proposalValidate.</t>
+        </is>
+      </c>
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>200 with validation result; bind succeeds when Vahan class matches.</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 500 MO-PLATFORM-COMMON-E9998 (generic). PCAR + MH12AB1234 bind gives 422 'VAHAN vehicle class M-Cycle/Scooter(2WN) does not match policy vehicle category 11'. Vahan GetVehicleData also returned 'wallet balance is low' intermittently.</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>traces 38dc9f05ff0b2d7b4900f289d5aa4489, be65b2fcf25079f76cf3081ff8793d1e, 1f55a3c08b388543bef93090c388d880</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="8" t="inlineStr">
+        <is>
+          <t>UAT-BUG-03</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="C4" s="8" t="inlineStr">
+        <is>
+          <t>A36.2 Upload claim document / A39.2 claim document tree</t>
+        </is>
+      </c>
+      <c r="D4" s="8" t="inlineStr">
+        <is>
+          <t>POST /api/platform/attachment-core/attachment/v1/uploadMulti ; POST .../getTreeData</t>
+        </is>
+      </c>
+      <c r="E4" s="8" t="inlineStr">
+        <is>
+          <t>Claim document types not configured; claim upload returns HTTP 500</t>
+        </is>
+      </c>
+      <c r="F4" s="8" t="inlineStr">
+        <is>
+          <t>1) Raise FNOL (e.g. PC-1204-26-00000001). 2) getTreeData BusinessType 001, ProductLine 01, ProductCode 1204. 3) uploadMulti BusinessType 001, Directory Motor_TP_01.</t>
+        </is>
+      </c>
+      <c r="G4" s="8" t="inlineStr">
+        <is>
+          <t>Tree lists Motor_TP_xx nodes; upload returns AttachFileId.</t>
+        </is>
+      </c>
+      <c r="H4" s="8" t="inlineStr">
+        <is>
+          <t>Tree has only BUSINESS_NO_ID and RECYCLE_ID; upload HTTP 500.</t>
+        </is>
+      </c>
+      <c r="I4" s="8" t="inlineStr">
+        <is>
+          <t>trace 0888b514a045b9cd704595b730e2f0fa (Motor_TP_01), 165b451daf84998da10dbaac3fa58b41 (01)</t>
+        </is>
+      </c>
+      <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="8" t="inlineStr">
+        <is>
+          <t>UAT-BUG-04</t>
+        </is>
+      </c>
+      <c r="B5" s="8" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="C5" s="8" t="inlineStr">
+        <is>
+          <t>Generic error handling (validate / bind / upload)</t>
+        </is>
+      </c>
+      <c r="D5" s="8" t="inlineStr">
+        <is>
+          <t>various</t>
+        </is>
+      </c>
+      <c r="E5" s="8" t="inlineStr">
+        <is>
+          <t>Unhandled exceptions return generic E9998 with no cause</t>
+        </is>
+      </c>
+      <c r="F5" s="8" t="inlineStr">
+        <is>
+          <t>See BUG-02 and BUG-03</t>
+        </is>
+      </c>
+      <c r="G5" s="8" t="inlineStr">
+        <is>
+          <t>Specific validation error (as bind returns for class mismatch).</t>
+        </is>
+      </c>
+      <c r="H5" s="8" t="inlineStr">
+        <is>
+          <t>Generic 'Exception has been thrown' message.</t>
+        </is>
+      </c>
+      <c r="I5" s="8" t="inlineStr">
+        <is>
+          <t>see traces above</t>
+        </is>
+      </c>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="8" t="inlineStr">
+        <is>
+          <t>UAT-OBS-05</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>A08.1 searchSCList</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>POST /api/platform/saleschannel/channel/searchSCList</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>Result depends on request shape: orInConditions ScStatus [1] returns Total 0; omitting it returns agents</t>
+        </is>
+      </c>
+      <c r="F6" s="8" t="inlineStr">
+        <is>
+          <t>Compare with and without searchCondition.orInConditions.ScStatus</t>
+        </is>
+      </c>
+      <c r="G6" s="8" t="inlineStr">
+        <is>
+          <t>Agents with status 1 returned.</t>
+        </is>
+      </c>
+      <c r="H6" s="8" t="inlineStr">
+        <is>
+          <t>Total 0 with ScStatus [1] (integer) filter.</t>
+        </is>
+      </c>
+      <c r="I6" s="8" t="inlineStr">
+        <is>
+          <t>new agent PTY00000000000003 appears only without the filter</t>
+        </is>
+      </c>
+      <c r="J6" s="8" t="inlineStr">
+        <is>
+          <t>Clarify spec</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="8" t="inlineStr">
+        <is>
+          <t>UAT-OBS-06</t>
+        </is>
+      </c>
+      <c r="B7" s="8" t="inlineStr">
+        <is>
+          <t>Info</t>
+        </is>
+      </c>
+      <c r="C7" s="8" t="inlineStr">
+        <is>
+          <t>A42.x FNOL</t>
+        </is>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
+        <is>
+          <t>POST .../ECS_business_fnol</t>
+        </is>
+      </c>
+      <c r="E7" s="8" t="inlineStr">
+        <is>
+          <t>Misleading message: loss date before policy start returns 'The policy does not exist!' (MO-Claim-Info-E0002)</t>
+        </is>
+      </c>
+      <c r="F7" s="8" t="inlineStr">
+        <is>
+          <t>FNOL with AccidentTime before policy EffectiveDate</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Message that the loss date is outside the cover period.</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>MO-Claim-Info-E0002 'The policy does not exist!'</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>PP-1005-26-00000052-00</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:K86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -5279,7 +5678,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9516,7 +9915,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9876,7 +10275,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -9961,7 +10360,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
Bugs grouped API-wise in UAT report and email draft
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_016KaHijVTfXKJr6MMzYd7aP
</commit_message>
<xml_diff>
--- a/Protec_UAT_API_Test_Report.xlsx
+++ b/Protec_UAT_API_Test_Report.xlsx
@@ -8,7 +8,7 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bugs" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bugs by API" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All APIs" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Success" sheetId="4" state="visible" r:id="rId4"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Failure" sheetId="5" state="visible" r:id="rId5"/>
@@ -16,6 +16,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Not tested" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Bugs by API'!$A$1:$L$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'All APIs'!$A$1:$K$86</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Success'!$A$1:$K$81</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Failure'!$A$1:$K$6</definedName>
@@ -46,7 +47,7 @@
       <color rgb="00FFFFFF"/>
     </font>
   </fonts>
-  <fills count="9">
+  <fills count="11">
     <fill>
       <patternFill/>
     </fill>
@@ -88,6 +89,16 @@
         <fgColor rgb="00C00000"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="1">
     <border>
@@ -101,7 +112,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -128,6 +139,15 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -774,68 +794,80 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J7"/>
+  <dimension ref="A1:L10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="30" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="50" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="50" customWidth="1" min="8" max="8"/>
-    <col width="44" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="46" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="52" customWidth="1" min="7" max="7"/>
+    <col width="56" customWidth="1" min="8" max="8"/>
+    <col width="34" customWidth="1" min="9" max="9"/>
+    <col width="52" customWidth="1" min="10" max="10"/>
+    <col width="44" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="13" t="inlineStr">
         <is>
+          <t>API No.</t>
+        </is>
+      </c>
+      <c r="B1" s="13" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="C1" s="13" t="inlineStr">
+        <is>
+          <t>Use case</t>
+        </is>
+      </c>
+      <c r="D1" s="13" t="inlineStr">
+        <is>
+          <t>Endpoint</t>
+        </is>
+      </c>
+      <c r="E1" s="13" t="inlineStr">
+        <is>
           <t>Bug ID</t>
         </is>
       </c>
-      <c r="B1" s="13" t="inlineStr">
+      <c r="F1" s="13" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="C1" s="13" t="inlineStr">
-        <is>
-          <t>API / use case</t>
-        </is>
-      </c>
-      <c r="D1" s="13" t="inlineStr">
-        <is>
-          <t>Endpoint</t>
-        </is>
-      </c>
-      <c r="E1" s="13" t="inlineStr">
-        <is>
-          <t>Summary</t>
-        </is>
-      </c>
-      <c r="F1" s="13" t="inlineStr">
+      <c r="G1" s="13" t="inlineStr">
+        <is>
+          <t>Issue</t>
+        </is>
+      </c>
+      <c r="H1" s="13" t="inlineStr">
         <is>
           <t>Steps to reproduce</t>
         </is>
       </c>
-      <c r="G1" s="13" t="inlineStr">
+      <c r="I1" s="13" t="inlineStr">
         <is>
           <t>Expected</t>
         </is>
       </c>
-      <c r="H1" s="13" t="inlineStr">
+      <c r="J1" s="13" t="inlineStr">
         <is>
           <t>Actual</t>
         </is>
       </c>
-      <c r="I1" s="13" t="inlineStr">
-        <is>
-          <t>Evidence (trace / policy / claim)</t>
-        </is>
-      </c>
-      <c r="J1" s="13" t="inlineStr">
+      <c r="K1" s="13" t="inlineStr">
+        <is>
+          <t>Evidence (trace / policy)</t>
+        </is>
+      </c>
+      <c r="L1" s="13" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
@@ -844,50 +876,60 @@
     <row r="2">
       <c r="A2" s="8" t="inlineStr">
         <is>
-          <t>UAT-BUG-01</t>
+          <t>A07</t>
         </is>
       </c>
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Vehicle data auto population</t>
         </is>
       </c>
       <c r="C2" s="8" t="inlineStr">
         <is>
-          <t>A31.1 proposalSendPrepayment (float issuance)</t>
+          <t>A07.1/A07.2</t>
         </is>
       </c>
       <c r="D2" s="8" t="inlineStr">
         <is>
-          <t>POST /api/protecuat/api-orchestration/v1/flow/agentPortal_proposalSendPrepayment</t>
+          <t>POST /api/protecuat/api-orchestration/v1/flow/GetVehicleData</t>
         </is>
       </c>
       <c r="E2" s="8" t="inlineStr">
         <is>
-          <t>Policy issued on float with NO float debit when underwriting result is a referral (AutoUwResultCode 2)</t>
-        </is>
-      </c>
-      <c r="F2" s="8" t="inlineStr">
-        <is>
-          <t>1) Agent PTY00000000000003 with float 532527. 2) Quote/bind PCAR with VehicleMake 1001 (UW referral) or PCV with RTO MH12. 3) Call proposalSendPrepayment with the bound PolicyObject.</t>
+          <t>UAT-BUG-05</t>
+        </is>
+      </c>
+      <c r="F2" s="14" t="inlineStr">
+        <is>
+          <t>Medium</t>
         </is>
       </c>
       <c r="G2" s="8" t="inlineStr">
         <is>
-          <t>Either float debited by DuePremium, or policy not issued until UW approves.</t>
+          <t>Intermittent Vahan failure: 'you are not authorized to make this request as your wallet balance is low'</t>
         </is>
       </c>
       <c r="H2" s="8" t="inlineStr">
         <is>
-          <t>Policy reaches ProposalStatus 3 (issued) and getCollectionTransHis shows no debit. Same PCAR with make 1002 (AutoUwResultCode 1) is debited 4473.38.</t>
+          <t>Call GetVehicleData for MH12XX0008 (Source Core, Stage Quote)</t>
         </is>
       </c>
       <c r="I2" s="8" t="inlineStr">
         <is>
-          <t>PP-1005-26-00000052-00 (4473.38) and PP-1202-26-00000027-00 (27358.30) not debited; PP-1005-26-00000053-00 debited</t>
+          <t>vehicle fields returned</t>
         </is>
       </c>
       <c r="J2" s="8" t="inlineStr">
+        <is>
+          <t>success=false, empty fields, response_message 'wallet balance is low' (seen 08:50-08:58; passed again later)</t>
+        </is>
+      </c>
+      <c r="K2" s="8" t="inlineStr">
+        <is>
+          <t>vahan ref ZOOP_MH12XX000820261028085031000</t>
+        </is>
+      </c>
+      <c r="L2" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -896,102 +938,122 @@
     <row r="3">
       <c r="A3" s="8" t="inlineStr">
         <is>
-          <t>UAT-BUG-02</t>
+          <t>A08</t>
         </is>
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Search sales channel (producers)</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
         <is>
-          <t>A27.1 proposalValidate / A29.1 proposalBind</t>
+          <t>A08.1</t>
         </is>
       </c>
       <c r="D3" s="8" t="inlineStr">
         <is>
-          <t>POST .../agentPortal_proposalValidate and .../agentPortal_proposalBind</t>
+          <t>POST /api/platform/saleschannel/channel/searchSCList</t>
         </is>
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
-          <t>HTTP 500 for registered vehicles (MH12AB1234, KA01AB1234); same proposals pass with MH12XX0008 or RegistrationNo NEW</t>
-        </is>
-      </c>
-      <c r="F3" s="8" t="inlineStr">
-        <is>
-          <t>1) Persist/calc/create/save/calc a P2W (or PCV/GCV) proposal with RegistrationNo MH12AB1234, ChannelType AP. 2) Call proposalValidate.</t>
+          <t>UAT-OBS-06</t>
+        </is>
+      </c>
+      <c r="F3" s="15" t="inlineStr">
+        <is>
+          <t>Info</t>
         </is>
       </c>
       <c r="G3" s="8" t="inlineStr">
         <is>
-          <t>200 with validation result; bind succeeds when Vahan class matches.</t>
+          <t>Returns Total 0 when searchCondition.orInConditions.ScStatus [1] is sent; agents are returned when the filter is omitted</t>
         </is>
       </c>
       <c r="H3" s="8" t="inlineStr">
         <is>
-          <t>HTTP 500 MO-PLATFORM-COMMON-E9998 (generic). PCAR + MH12AB1234 bind gives 422 'VAHAN vehicle class M-Cycle/Scooter(2WN) does not match policy vehicle category 11'. Vahan GetVehicleData also returned 'wallet balance is low' intermittently.</t>
+          <t>Search PCAR with and without orInConditions ScStatus</t>
         </is>
       </c>
       <c r="I3" s="8" t="inlineStr">
         <is>
-          <t>traces 38dc9f05ff0b2d7b4900f289d5aa4489, be65b2fcf25079f76cf3081ff8793d1e, 1f55a3c08b388543bef93090c388d880</t>
+          <t>Active agents returned in both cases</t>
         </is>
       </c>
       <c r="J3" s="8" t="inlineStr">
         <is>
-          <t>Open</t>
+          <t>Total 0 with ScStatus [1]</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>agent PTY00000000000003</t>
+        </is>
+      </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>Clarify spec</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="8" t="inlineStr">
         <is>
-          <t>UAT-BUG-03</t>
+          <t>A27</t>
         </is>
       </c>
       <c r="B4" s="8" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>Proposal validate</t>
         </is>
       </c>
       <c r="C4" s="8" t="inlineStr">
         <is>
-          <t>A36.2 Upload claim document / A39.2 claim document tree</t>
+          <t>A27.1</t>
         </is>
       </c>
       <c r="D4" s="8" t="inlineStr">
         <is>
-          <t>POST /api/platform/attachment-core/attachment/v1/uploadMulti ; POST .../getTreeData</t>
+          <t>POST /api/protecuat/api-orchestration/v1/flow/agentPortal_proposalValidate</t>
         </is>
       </c>
       <c r="E4" s="8" t="inlineStr">
         <is>
-          <t>Claim document types not configured; claim upload returns HTTP 500</t>
-        </is>
-      </c>
-      <c r="F4" s="8" t="inlineStr">
-        <is>
-          <t>1) Raise FNOL (e.g. PC-1204-26-00000001). 2) getTreeData BusinessType 001, ProductLine 01, ProductCode 1204. 3) uploadMulti BusinessType 001, Directory Motor_TP_01.</t>
+          <t>UAT-BUG-02</t>
+        </is>
+      </c>
+      <c r="F4" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="G4" s="8" t="inlineStr">
         <is>
-          <t>Tree lists Motor_TP_xx nodes; upload returns AttachFileId.</t>
+          <t>HTTP 500 for registered vehicles (MH12AB1234, KA01AB1234); passes for MH12XX0008 and RegistrationNo NEW</t>
         </is>
       </c>
       <c r="H4" s="8" t="inlineStr">
         <is>
-          <t>Tree has only BUSINESS_NO_ID and RECYCLE_ID; upload HTTP 500.</t>
+          <t>Persist/calc/create/save/calc a P2W/PCV/GCV proposal with RegistrationNo MH12AB1234, ChannelType AP; call proposalValidate</t>
         </is>
       </c>
       <c r="I4" s="8" t="inlineStr">
         <is>
-          <t>trace 0888b514a045b9cd704595b730e2f0fa (Motor_TP_01), 165b451daf84998da10dbaac3fa58b41 (01)</t>
+          <t>200 with validation result</t>
         </is>
       </c>
       <c r="J4" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 500 MO-PLATFORM-COMMON-E9998 (generic)</t>
+        </is>
+      </c>
+      <c r="K4" s="8" t="inlineStr">
+        <is>
+          <t>38dc9f05ff0b2d7b4900f289d5aa4489</t>
+        </is>
+      </c>
+      <c r="L4" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1000,50 +1062,60 @@
     <row r="5">
       <c r="A5" s="8" t="inlineStr">
         <is>
-          <t>UAT-BUG-04</t>
+          <t>A29</t>
         </is>
       </c>
       <c r="B5" s="8" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>Proposal bind</t>
         </is>
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>Generic error handling (validate / bind / upload)</t>
+          <t>A29.1</t>
         </is>
       </c>
       <c r="D5" s="8" t="inlineStr">
         <is>
-          <t>various</t>
+          <t>POST /api/protecuat/api-orchestration/v1/flow/agentPortal_proposalBind</t>
         </is>
       </c>
       <c r="E5" s="8" t="inlineStr">
         <is>
-          <t>Unhandled exceptions return generic E9998 with no cause</t>
-        </is>
-      </c>
-      <c r="F5" s="8" t="inlineStr">
-        <is>
-          <t>See BUG-02 and BUG-03</t>
+          <t>UAT-BUG-02</t>
+        </is>
+      </c>
+      <c r="F5" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="G5" s="8" t="inlineStr">
         <is>
-          <t>Specific validation error (as bind returns for class mismatch).</t>
+          <t>HTTP 500 for registered vehicles; PCAR + MH12AB1234 gives 422 class mismatch instead (inconsistent behaviour)</t>
         </is>
       </c>
       <c r="H5" s="8" t="inlineStr">
         <is>
-          <t>Generic 'Exception has been thrown' message.</t>
+          <t>Bind the proposal from A27 repro</t>
         </is>
       </c>
       <c r="I5" s="8" t="inlineStr">
         <is>
-          <t>see traces above</t>
+          <t>Bound PolicyObject</t>
         </is>
       </c>
       <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>P2W/PCV/GCV: HTTP 500; PCAR: 422 'VAHAN vehicle class M-Cycle/Scooter(2WN) does not match policy vehicle category 11'</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>be65b2fcf25079f76cf3081ff8793d1e (500); 1f55a3c08b388543bef93090c388d880 (422)</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -1052,108 +1124,315 @@
     <row r="6">
       <c r="A6" s="8" t="inlineStr">
         <is>
-          <t>UAT-OBS-05</t>
+          <t>A31</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Proposal send prepayment (float issuance)</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>A08.1 searchSCList</t>
+          <t>A31.1</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>POST /api/platform/saleschannel/channel/searchSCList</t>
+          <t>POST /api/protecuat/api-orchestration/v1/flow/agentPortal_proposalSendPrepayment</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>Result depends on request shape: orInConditions ScStatus [1] returns Total 0; omitting it returns agents</t>
-        </is>
-      </c>
-      <c r="F6" s="8" t="inlineStr">
-        <is>
-          <t>Compare with and without searchCondition.orInConditions.ScStatus</t>
+          <t>UAT-BUG-01</t>
+        </is>
+      </c>
+      <c r="F6" s="12" t="inlineStr">
+        <is>
+          <t>High</t>
         </is>
       </c>
       <c r="G6" s="8" t="inlineStr">
         <is>
-          <t>Agents with status 1 returned.</t>
+          <t>Policy issued with NO float debit when underwriting result is a referral (AutoUwResultCode 2)</t>
         </is>
       </c>
       <c r="H6" s="8" t="inlineStr">
         <is>
-          <t>Total 0 with ScStatus [1] (integer) filter.</t>
+          <t>Agent with funded float; bind PCAR with VehicleMake 1001 or PCV with RTO MH12; call proposalSendPrepayment with the bound PolicyObject</t>
         </is>
       </c>
       <c r="I6" s="8" t="inlineStr">
         <is>
-          <t>new agent PTY00000000000003 appears only without the filter</t>
+          <t>Float debited by DuePremium, or policy not issued until UW approves</t>
         </is>
       </c>
       <c r="J6" s="8" t="inlineStr">
         <is>
-          <t>Clarify spec</t>
+          <t>ProposalStatus 3 (issued); getCollectionTransHis shows no debit. Same PCAR with make 1002 (AutoUwResultCode 1) is debited 4473.38</t>
+        </is>
+      </c>
+      <c r="K6" s="8" t="inlineStr">
+        <is>
+          <t>PP-1005-26-00000052-00 (4473.38), PP-1202-26-00000027-00 (27358.30) not debited; PP-1005-26-00000053-00 debited</t>
+        </is>
+      </c>
+      <c r="L6" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="8" t="inlineStr">
         <is>
-          <t>UAT-OBS-06</t>
+          <t>A36</t>
         </is>
       </c>
       <c r="B7" s="8" t="inlineStr">
         <is>
-          <t>Info</t>
+          <t>Upload document (claim)</t>
         </is>
       </c>
       <c r="C7" s="8" t="inlineStr">
         <is>
-          <t>A42.x FNOL</t>
+          <t>A36.2</t>
         </is>
       </c>
       <c r="D7" s="8" t="inlineStr">
         <is>
-          <t>POST .../ECS_business_fnol</t>
+          <t>POST /api/platform/attachment-core/attachment/v1/uploadMulti</t>
         </is>
       </c>
       <c r="E7" s="8" t="inlineStr">
         <is>
+          <t>UAT-BUG-03</t>
+        </is>
+      </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G7" s="8" t="inlineStr">
+        <is>
+          <t>Claim document upload returns HTTP 500</t>
+        </is>
+      </c>
+      <c r="H7" s="8" t="inlineStr">
+        <is>
+          <t>FNOL (e.g. PC-1204-26-00000001); uploadMulti BusinessType 001, BusinessNo claim no, Directory Motor_TP_01 (also 01)</t>
+        </is>
+      </c>
+      <c r="I7" s="8" t="inlineStr">
+        <is>
+          <t>AttachFileId returned</t>
+        </is>
+      </c>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>HTTP 500 MO-PLATFORM-COMMON-E9998</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>0888b514a045b9cd704595b730e2f0fa; 165b451daf84998da10dbaac3fa58b41</t>
+        </is>
+      </c>
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="8" t="inlineStr">
+        <is>
+          <t>A39</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>Document type tree (claim)</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>A39.2</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>POST /api/platform/attachment-core/attachment/v1/getTreeData</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>UAT-BUG-03</t>
+        </is>
+      </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="G8" s="8" t="inlineStr">
+        <is>
+          <t>Claim document types (Motor_TP_xx) not configured in UAT</t>
+        </is>
+      </c>
+      <c r="H8" s="8" t="inlineStr">
+        <is>
+          <t>getTreeData BusinessType 001, ProductLine 01, ProductCode 1204/1106/1202/1005</t>
+        </is>
+      </c>
+      <c r="I8" s="8" t="inlineStr">
+        <is>
+          <t>Motor_TP_xx nodes listed</t>
+        </is>
+      </c>
+      <c r="J8" s="8" t="inlineStr">
+        <is>
+          <t>Only BUSINESS_NO_ID and RECYCLE_ID nodes</t>
+        </is>
+      </c>
+      <c r="K8" s="8" t="inlineStr">
+        <is>
+          <t>claims PC-1204-26-00000001, PC-1106-26-00000001, PC-1202-26-00000001</t>
+        </is>
+      </c>
+      <c r="L8" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="8" t="inlineStr">
+        <is>
+          <t>A42</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="inlineStr">
+        <is>
+          <t>Submit FNOL</t>
+        </is>
+      </c>
+      <c r="C9" s="8" t="inlineStr">
+        <is>
+          <t>A42.1-A42.3</t>
+        </is>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
+        <is>
+          <t>POST /api/protecuat/api-orchestration/v1/flow/ECS_business_fnol</t>
+        </is>
+      </c>
+      <c r="E9" s="8" t="inlineStr">
+        <is>
+          <t>UAT-OBS-07</t>
+        </is>
+      </c>
+      <c r="F9" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G9" s="8" t="inlineStr">
+        <is>
           <t>Misleading message: loss date before policy start returns 'The policy does not exist!' (MO-Claim-Info-E0002)</t>
         </is>
       </c>
-      <c r="F7" s="8" t="inlineStr">
-        <is>
-          <t>FNOL with AccidentTime before policy EffectiveDate</t>
-        </is>
-      </c>
-      <c r="G7" s="8" t="inlineStr">
-        <is>
-          <t>Message that the loss date is outside the cover period.</t>
-        </is>
-      </c>
-      <c r="H7" s="8" t="inlineStr">
+      <c r="H9" s="8" t="inlineStr">
+        <is>
+          <t>FNOL with AccidentTime earlier than the policy EffectiveDate</t>
+        </is>
+      </c>
+      <c r="I9" s="8" t="inlineStr">
+        <is>
+          <t>Message that the loss date is outside the cover period</t>
+        </is>
+      </c>
+      <c r="J9" s="8" t="inlineStr">
         <is>
           <t>MO-Claim-Info-E0002 'The policy does not exist!'</t>
         </is>
       </c>
-      <c r="I7" s="8" t="inlineStr">
+      <c r="K9" s="8" t="inlineStr">
         <is>
           <t>PP-1005-26-00000052-00</t>
         </is>
       </c>
-      <c r="J7" s="8" t="inlineStr">
+      <c r="L9" s="8" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>All</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>Error handling (A27, A29, A36)</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>various</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>UAT-BUG-04</t>
+        </is>
+      </c>
+      <c r="F10" s="16" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Unhandled exceptions return a generic E9998 message with no cause</t>
+        </is>
+      </c>
+      <c r="H10" s="8" t="inlineStr">
+        <is>
+          <t>See BUG-02, BUG-03</t>
+        </is>
+      </c>
+      <c r="I10" s="8" t="inlineStr">
+        <is>
+          <t>Specific validation message (as bind returns for class mismatch)</t>
+        </is>
+      </c>
+      <c r="J10" s="8" t="inlineStr">
+        <is>
+          <t>'Exception has been thrown, check it in logging system...'</t>
+        </is>
+      </c>
+      <c r="K10" s="8" t="inlineStr">
+        <is>
+          <t>traces above</t>
+        </is>
+      </c>
+      <c r="L10" s="8" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
+  <autoFilter ref="A1:L10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>